<commit_message>
chore: actualizar next-env.d.ts, tsconfig.tsbuildinfo y excel de productos
</commit_message>
<xml_diff>
--- a/public/PRODUCTOS PÁGINA WEB.xlsx
+++ b/public/PRODUCTOS PÁGINA WEB.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/e23cdc8a63c7ec0a/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Electro-Thina\public\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="2" documentId="8_{40038D52-8EEE-4689-9B9F-BE52DADDF488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{53792695-3577-4D7E-A5BB-A3E29367FEF4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9B2E68D-102E-4023-B7B1-5D2623A17075}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{4B16B4B7-6DA1-49A3-8375-87E5A1424D06}"/>
   </bookViews>
@@ -736,300 +736,12 @@
         </r>
       </text>
     </comment>
-    <comment ref="C58" authorId="0" shapeId="0" xr:uid="{CCE2A19B-2EEB-46D4-A059-810F878BBD62}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-VARIAS MEDIDAS MISMO MODELO SOLO VARIA EL TAMAÑO</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C59" authorId="0" shapeId="0" xr:uid="{2A1DAF71-AD54-45A2-A767-C81FD7E40CD1}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-VARIAS MEDIDAS MISMO MODELO SOLO VARIA EL TAMAÑO</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C60" authorId="0" shapeId="0" xr:uid="{164CAEAA-D5BA-4839-A93E-1AFDA2032A22}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-VARIAS MEDIDAS MISMO MODELO SOLO VARIA EL TAMAÑO</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C61" authorId="0" shapeId="0" xr:uid="{B4C87F76-BBFE-4F62-A585-FC26D3194EBD}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-DOS MEDIDAS MISMO MODELO DIFERENTES MARCAS</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C64" authorId="0" shapeId="0" xr:uid="{DB16F56E-0C86-4366-9848-F4434CD0E62F}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-TIENE DOS MEDIDAS </t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C67" authorId="0" shapeId="0" xr:uid="{2AF77EE5-39C8-4D8C-9480-6C5ACCED70B8}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-DOS MEDIDAS</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C68" authorId="0" shapeId="0" xr:uid="{ED195B14-AA0D-4564-9A54-500C191579E3}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-VARIAS MEDIDAS MISMO MODELO </t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C69" authorId="0" shapeId="0" xr:uid="{2FCE7671-B721-4208-B3BE-97ADC0C038B1}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-DOS MEDIDAS MISMO MODELO</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C70" authorId="0" shapeId="0" xr:uid="{B20506B9-0914-40FE-87D1-9B828DBF2D16}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-DOS MEDIDAS MISMO MODELO </t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C71" authorId="0" shapeId="0" xr:uid="{CEC4A62B-B861-40C2-B02E-E7562C9D3BC3}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-DOS MEDIDAS</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C72" authorId="0" shapeId="0" xr:uid="{3F78DBC9-BF14-4944-8E66-BC315011CB90}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-VARIAS MEDIDAS</t>
-        </r>
-      </text>
-    </comment>
-    <comment ref="C74" authorId="0" shapeId="0" xr:uid="{75887068-A812-4E42-AE10-00BA29533992}">
-      <text>
-        <r>
-          <rPr>
-            <b/>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t>ALEXZA CORPORACION:</t>
-        </r>
-        <r>
-          <rPr>
-            <sz val="9"/>
-            <color indexed="81"/>
-            <rFont val="Tahoma"/>
-            <family val="2"/>
-          </rPr>
-          <t xml:space="preserve">
-VARIAS MEDIDAS MISMO MODELO </t>
-        </r>
-      </text>
-    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="106">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="103" uniqueCount="72">
   <si>
     <t>PRODUCTO</t>
   </si>
@@ -1190,90 +902,15 @@
     <t>GRAPA FORJADA DE 3/8</t>
   </si>
   <si>
-    <t>GRAPA PARALELA DOS VIAS 3 PERNO PESADA</t>
-  </si>
-  <si>
-    <t>GRAPA PARALELA DOS VIAS 2 PERNO PESADA</t>
-  </si>
-  <si>
-    <t>GRAPA PARALELA UNA VIA 2 PERNO PESADA</t>
-  </si>
-  <si>
-    <t>GRILLETE FORJADO DE 1/2 PIN ROJO</t>
-  </si>
-  <si>
-    <t>GUARDACABLE DE 3/8</t>
-  </si>
-  <si>
-    <t>GUARDACABO DE 3/8 DE RETENIDA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">HEBILLA DE ACERO INOXIDABLE </t>
-  </si>
-  <si>
-    <t>KIT DE HUESO COMPLETO</t>
-  </si>
-  <si>
-    <t>MASTIL PARA TORRE</t>
-  </si>
-  <si>
-    <t>PARARRAYO TETRAPUNTAL TIPO FRNKLIN 1/2 C/BASE</t>
-  </si>
-  <si>
-    <t>PASTORAL DE FG 1 1 /4 X 1.50 MTS</t>
-  </si>
-  <si>
-    <t>PERNO COCHE DE A°G° 1/2Ø X 6" DE LONG CON TUERCA</t>
-  </si>
-  <si>
-    <t>TEMPLADOR TIPO SAPITO MONOFASICO</t>
-  </si>
-  <si>
-    <t>TERMINAL A COMPRESION DE 10MM C/ LARGO</t>
-  </si>
-  <si>
-    <t>TEMPLADOR FORJADO OJO / GANCHO DE 1/2</t>
-  </si>
-  <si>
-    <t>TEMPLADOR FORJADO OJO / OJO DE 1/2</t>
-  </si>
-  <si>
-    <t>TEMPLADOR OJO / GANCHO DE A°G° DE 5/8X10''</t>
-  </si>
-  <si>
-    <t>TUBO BASTON DE A°G° 2 X 3MTS</t>
-  </si>
-  <si>
-    <t>TIMBLER CLEVIS GUARDACABO HORQUILLA AL</t>
-  </si>
-  <si>
-    <t>VARILLA DE COBRE 5/8X2.40 MTS</t>
-  </si>
-  <si>
     <t xml:space="preserve">VARILLAS </t>
   </si>
   <si>
-    <t xml:space="preserve">ACOMETIDA </t>
-  </si>
-  <si>
     <t>FIBRA ÓPTICA</t>
   </si>
   <si>
-    <t>TEMPLADORES</t>
-  </si>
-  <si>
-    <t>TERMINALES</t>
-  </si>
-  <si>
-    <t>SOPORTE PASANTE ADSS</t>
-  </si>
-  <si>
     <t>PERNOS</t>
   </si>
   <si>
-    <t>ILUMINACIÓN</t>
-  </si>
-  <si>
     <t>PARARRAYOS</t>
   </si>
   <si>
@@ -1283,24 +920,9 @@
     <t>GRAPAS</t>
   </si>
   <si>
-    <t>GRILLETES</t>
-  </si>
-  <si>
-    <t>HEBILLAS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ANCLAJES </t>
-  </si>
-  <si>
     <t>ESPIGAS</t>
   </si>
   <si>
-    <t>ENLACE METALICO</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SECCIONADORES </t>
-  </si>
-  <si>
     <t>FUSIBLES</t>
   </si>
   <si>
@@ -1319,22 +941,10 @@
     <t>ADAPTADORES</t>
   </si>
   <si>
-    <t>CEMENTO CONDUCTIVO X 25 KILOS TERRAWELD</t>
-  </si>
-  <si>
     <t>CINTAS</t>
   </si>
   <si>
     <t>RETENIDAS</t>
-  </si>
-  <si>
-    <t>CAJA DE REGISTRO TIPO BALDE DE PVC PARA PUESTA A TIERRA</t>
-  </si>
-  <si>
-    <t>ARMELLA TIRAFON DE A°G°</t>
-  </si>
-  <si>
-    <t>BENTONITA SODICA X 30KG</t>
   </si>
   <si>
     <t xml:space="preserve">AMARRES </t>
@@ -1389,18 +999,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="3">
@@ -1443,26 +1047,17 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1481,9 +1076,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Tema de Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - Tema de 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -1521,7 +1116,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -1627,7 +1222,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -1769,7 +1364,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -1777,7 +1372,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4937413E-5D3C-4560-BE0B-2D699E135A37}">
-  <dimension ref="B4:G80"/>
+  <dimension ref="B4:G54"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="68.42578125" customWidth="1"/>
@@ -1789,481 +1384,481 @@
       <c r="B4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="12" t="s">
+      <c r="C4" s="3" t="s">
         <v>0</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="G4" s="4"/>
+      <c r="G4" s="2"/>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B5" s="1">
         <v>1</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="4" t="s">
         <v>2</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B6" s="1">
         <v>2</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="4" t="s">
         <v>3</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B7" s="1">
         <v>3</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="4" t="s">
         <v>4</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>93</v>
+        <v>63</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B8" s="1">
         <v>4</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="4" t="s">
         <v>5</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>93</v>
+        <v>63</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B9" s="1">
         <v>5</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="4" t="s">
         <v>6</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>93</v>
+        <v>63</v>
       </c>
     </row>
     <row r="10" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B10" s="1">
         <v>6</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="4" t="s">
         <v>7</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>93</v>
+        <v>63</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B11" s="1">
         <v>7</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="4" t="s">
         <v>8</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>93</v>
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B12" s="1">
         <v>8</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="4" t="s">
         <v>10</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
     </row>
     <row r="13" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B13" s="1">
         <v>9</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>11</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="1">
         <v>10</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>12</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
     </row>
     <row r="15" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B15" s="1">
         <v>11</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>13</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
     </row>
     <row r="16" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B16" s="1">
         <v>12</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="4" t="s">
         <v>14</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>91</v>
+        <v>61</v>
       </c>
     </row>
     <row r="17" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B17" s="1">
         <v>13</v>
       </c>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>15</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>104</v>
+        <v>70</v>
       </c>
     </row>
     <row r="18" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B18" s="1">
         <v>14</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>104</v>
+        <v>70</v>
       </c>
     </row>
     <row r="19" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B19" s="1">
         <v>15</v>
       </c>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>17</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>73</v>
+        <v>53</v>
       </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B20" s="1">
         <v>16</v>
       </c>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="4" t="s">
         <v>18</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>82</v>
+        <v>57</v>
       </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B21" s="1">
         <v>17</v>
       </c>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="4" t="s">
         <v>19</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>105</v>
+        <v>71</v>
       </c>
     </row>
     <row r="22" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B22" s="1">
         <v>18</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="4" t="s">
         <v>20</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>105</v>
+        <v>71</v>
       </c>
     </row>
     <row r="23" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B23" s="1">
         <v>19</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="4" t="s">
         <v>21</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B24" s="1">
         <v>20</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="4" t="s">
         <v>22</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>79</v>
+        <v>55</v>
       </c>
     </row>
     <row r="25" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B25" s="1">
         <v>21</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="4" t="s">
         <v>23</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>81</v>
+        <v>56</v>
       </c>
     </row>
     <row r="26" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B26" s="1">
         <v>22</v>
       </c>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="4" t="s">
         <v>24</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>94</v>
+        <v>64</v>
       </c>
     </row>
     <row r="27" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B27" s="1">
         <v>23</v>
       </c>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="4" t="s">
         <v>25</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>102</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B28" s="1">
         <v>24</v>
       </c>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="4" t="s">
         <v>26</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>73</v>
+        <v>53</v>
       </c>
     </row>
     <row r="29" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B29" s="1">
         <v>25</v>
       </c>
-      <c r="C29" s="9" t="s">
+      <c r="C29" s="5" t="s">
         <v>27</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
     </row>
     <row r="30" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B30" s="1">
         <v>26</v>
       </c>
-      <c r="C30" s="10" t="s">
+      <c r="C30" s="5" t="s">
         <v>28</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
     </row>
     <row r="31" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B31" s="1">
         <v>27</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="5" t="s">
         <v>29</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B32" s="1">
         <v>28</v>
       </c>
-      <c r="C32" s="10" t="s">
+      <c r="C32" s="5" t="s">
         <v>30</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
     </row>
     <row r="33" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B33" s="1">
         <v>29</v>
       </c>
-      <c r="C33" s="10" t="s">
+      <c r="C33" s="5" t="s">
         <v>31</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
     </row>
     <row r="34" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B34" s="1">
         <v>30</v>
       </c>
-      <c r="C34" s="9" t="s">
+      <c r="C34" s="5" t="s">
         <v>32</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
     </row>
     <row r="35" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B35" s="1">
         <v>31</v>
       </c>
-      <c r="C35" s="9" t="s">
+      <c r="C35" s="5" t="s">
         <v>33</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>103</v>
+        <v>69</v>
       </c>
     </row>
     <row r="36" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B36" s="1">
         <v>32</v>
       </c>
-      <c r="C36" s="10" t="s">
+      <c r="C36" s="5" t="s">
         <v>34</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
     </row>
     <row r="37" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B37" s="1">
         <v>33</v>
       </c>
-      <c r="C37" s="10" t="s">
+      <c r="C37" s="5" t="s">
         <v>35</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
     </row>
     <row r="38" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B38" s="1">
         <v>34</v>
       </c>
-      <c r="C38" s="10" t="s">
+      <c r="C38" s="5" t="s">
         <v>36</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
     </row>
     <row r="39" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B39" s="1">
         <v>35</v>
       </c>
-      <c r="C39" s="10" t="s">
+      <c r="C39" s="5" t="s">
         <v>37</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>95</v>
+        <v>65</v>
       </c>
     </row>
     <row r="40" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B40" s="1">
         <v>36</v>
       </c>
-      <c r="C40" s="10" t="s">
+      <c r="C40" s="5" t="s">
         <v>38</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>98</v>
+        <v>67</v>
       </c>
     </row>
     <row r="41" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B41" s="1">
         <v>37</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="5" t="s">
         <v>39</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>97</v>
+        <v>66</v>
       </c>
     </row>
     <row r="42" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B42" s="1">
         <v>38</v>
       </c>
-      <c r="C42" s="9" t="s">
+      <c r="C42" s="5" t="s">
         <v>40</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>82</v>
+        <v>57</v>
       </c>
     </row>
     <row r="43" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B43" s="1">
         <v>39</v>
       </c>
-      <c r="C43" s="9" t="s">
+      <c r="C43" s="5" t="s">
         <v>41</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>93</v>
+        <v>63</v>
       </c>
     </row>
     <row r="44" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B44" s="1">
         <v>40</v>
       </c>
-      <c r="C44" s="11" t="s">
+      <c r="C44" s="5" t="s">
         <v>42</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>75</v>
+        <v>54</v>
       </c>
     </row>
     <row r="45" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B45" s="1">
         <v>41</v>
       </c>
-      <c r="C45" s="9" t="s">
+      <c r="C45" s="5" t="s">
         <v>43</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>91</v>
+        <v>61</v>
       </c>
     </row>
     <row r="46" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B46" s="1">
         <v>42</v>
       </c>
-      <c r="C46" s="9" t="s">
+      <c r="C46" s="5" t="s">
         <v>44</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>92</v>
+        <v>62</v>
       </c>
     </row>
     <row r="47" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B47" s="1">
         <v>43</v>
       </c>
-      <c r="C47" s="10" t="s">
+      <c r="C47" s="5" t="s">
         <v>45</v>
       </c>
       <c r="D47" s="1" t="s">
@@ -2274,285 +1869,77 @@
       <c r="B48" s="1">
         <v>44</v>
       </c>
-      <c r="C48" s="9" t="s">
+      <c r="C48" s="5" t="s">
         <v>46</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
     </row>
     <row r="49" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B49" s="1">
         <v>45</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="C49" s="5" t="s">
         <v>47</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
     </row>
     <row r="50" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B50" s="1">
         <v>46</v>
       </c>
-      <c r="C50" s="10" t="s">
+      <c r="C50" s="5" t="s">
         <v>48</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>87</v>
+        <v>59</v>
       </c>
     </row>
     <row r="51" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B51" s="1">
         <v>47</v>
       </c>
-      <c r="C51" s="9" t="s">
+      <c r="C51" s="5" t="s">
         <v>49</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>90</v>
+        <v>60</v>
       </c>
     </row>
     <row r="52" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B52" s="1">
         <v>48</v>
       </c>
-      <c r="C52" s="9" t="s">
+      <c r="C52" s="5" t="s">
         <v>50</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
     </row>
     <row r="53" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B53" s="1">
         <v>49</v>
       </c>
-      <c r="C53" s="9" t="s">
+      <c r="C53" s="5" t="s">
         <v>51</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>83</v>
+        <v>58</v>
       </c>
     </row>
     <row r="54" spans="2:4" x14ac:dyDescent="0.25">
       <c r="B54" s="1">
         <v>50</v>
       </c>
-      <c r="C54" s="9" t="s">
+      <c r="C54" s="5" t="s">
         <v>52</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="55" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C55" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="D55" s="8" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="56" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C56" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="D56" s="8" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="57" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C57" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="D57" s="8" t="s">
-        <v>83</v>
-      </c>
-    </row>
-    <row r="58" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C58" s="6" t="s">
-        <v>56</v>
-      </c>
-      <c r="D58" s="8" t="s">
-        <v>84</v>
-      </c>
-    </row>
-    <row r="59" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C59" s="6" t="s">
-        <v>57</v>
-      </c>
-      <c r="D59" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="60" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C60" s="6" t="s">
         <v>58</v>
-      </c>
-      <c r="D60" s="8" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="61" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C61" s="6" t="s">
-        <v>59</v>
-      </c>
-      <c r="D61" s="8" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="62" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C62" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="D62" s="8" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="63" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C63" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="D63" s="8" t="s">
-        <v>82</v>
-      </c>
-    </row>
-    <row r="64" spans="2:4" x14ac:dyDescent="0.25">
-      <c r="C64" s="6" t="s">
-        <v>62</v>
-      </c>
-      <c r="D64" s="8" t="s">
-        <v>81</v>
-      </c>
-    </row>
-    <row r="65" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C65" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="D65" s="8" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="66" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C66" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="D66" s="8" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="67" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C67" s="6" t="s">
-        <v>65</v>
-      </c>
-      <c r="D67" s="8" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="68" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C68" s="6" t="s">
-        <v>66</v>
-      </c>
-      <c r="D68" s="8" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="69" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C69" s="6" t="s">
-        <v>67</v>
-      </c>
-      <c r="D69" s="8" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="70" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C70" s="6" t="s">
-        <v>68</v>
-      </c>
-      <c r="D70" s="8" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="71" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C71" s="6" t="s">
-        <v>69</v>
-      </c>
-      <c r="D71" s="8" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="72" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C72" s="6" t="s">
-        <v>70</v>
-      </c>
-      <c r="D72" s="8" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="73" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C73" s="5" t="s">
-        <v>71</v>
-      </c>
-      <c r="D73" s="8" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="74" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C74" s="6" t="s">
-        <v>72</v>
-      </c>
-      <c r="D74" s="8" t="s">
-        <v>73</v>
-      </c>
-    </row>
-    <row r="75" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C75" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="D75" s="8" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="76" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C76" s="5" t="s">
-        <v>88</v>
-      </c>
-      <c r="D76" s="8" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="77" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C77" s="7" t="s">
-        <v>96</v>
-      </c>
-      <c r="D77" s="8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="78" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C78" s="5" t="s">
-        <v>99</v>
-      </c>
-      <c r="D78" s="8" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="79" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C79" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="D79" s="8" t="s">
-        <v>79</v>
-      </c>
-    </row>
-    <row r="80" spans="3:4" x14ac:dyDescent="0.25">
-      <c r="C80" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="D80" s="8" t="s">
-        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>